<commit_message>
Add net weight column to Fired Up OOCU5773452 HS code summary
Net weights per HS code taken from packing list 0055; total 6,795.7 kg
reconciles with the packing list N.W. total.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DEStrPTYqhj9hDeddsySih
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Fired_Up_OOCU5773452.xlsx
+++ b/output/HS_Code_Summary_Fired_Up_OOCU5773452.xlsx
@@ -515,16 +515,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -636,20 +637,25 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
+          <t>Net weight (kg)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
           <t>Gross weight (kg)</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Customs value (RMB)</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Antidumping</t>
         </is>
@@ -670,17 +676,20 @@
         <v>972</v>
       </c>
       <c r="D12" s="6" t="n">
+        <v>769.5</v>
+      </c>
+      <c r="E12" s="6" t="n">
         <v>834.3</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="F12" s="5" t="n">
         <v>59292</v>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -697,17 +706,20 @@
         <v>1662</v>
       </c>
       <c r="D13" s="9" t="n">
+        <v>1590</v>
+      </c>
+      <c r="E13" s="9" t="n">
         <v>1698.1</v>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="F13" s="8" t="n">
         <v>157728</v>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr"/>
+      <c r="H13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -724,17 +736,20 @@
         <v>168</v>
       </c>
       <c r="D14" s="6" t="n">
+        <v>99</v>
+      </c>
+      <c r="E14" s="6" t="n">
         <v>104.5</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="F14" s="5" t="n">
         <v>17808</v>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -751,17 +766,20 @@
         <v>156</v>
       </c>
       <c r="D15" s="9" t="n">
+        <v>221</v>
+      </c>
+      <c r="E15" s="9" t="n">
         <v>234</v>
       </c>
-      <c r="E15" s="8" t="n">
+      <c r="F15" s="8" t="n">
         <v>13728</v>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -778,17 +796,20 @@
         <v>1548</v>
       </c>
       <c r="D16" s="6" t="n">
+        <v>2868.1</v>
+      </c>
+      <c r="E16" s="6" t="n">
         <v>3033.3</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="F16" s="5" t="n">
         <v>83620</v>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>No*</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -805,17 +826,20 @@
         <v>250</v>
       </c>
       <c r="D17" s="12" t="n">
+        <v>287.5</v>
+      </c>
+      <c r="E17" s="12" t="n">
         <v>302.5</v>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="F17" s="11" t="n">
         <v>8875</v>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="G17" s="10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="H17" s="10" t="inlineStr">
         <is>
           <t>Yes - verify</t>
         </is>
@@ -836,17 +860,20 @@
         <v>360</v>
       </c>
       <c r="D18" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="E18" s="6" t="n">
         <v>50.4</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="F18" s="5" t="n">
         <v>9000</v>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -863,17 +890,20 @@
         <v>400</v>
       </c>
       <c r="D19" s="9" t="n">
+        <v>760</v>
+      </c>
+      <c r="E19" s="9" t="n">
         <v>820</v>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="F19" s="8" t="n">
         <v>15600</v>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -890,17 +920,20 @@
         <v>120</v>
       </c>
       <c r="D20" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="E20" s="6" t="n">
         <v>158</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="F20" s="5" t="n">
         <v>5520</v>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -917,17 +950,20 @@
         <v>30</v>
       </c>
       <c r="D21" s="9" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E21" s="9" t="n">
         <v>2.9</v>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="F21" s="8" t="n">
         <v>240</v>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr"/>
+      <c r="H21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
@@ -940,13 +976,16 @@
         <v>5666</v>
       </c>
       <c r="D22" s="15" t="n">
+        <v>6795.7</v>
+      </c>
+      <c r="E22" s="15" t="n">
         <v>7238</v>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="F22" s="14" t="n">
         <v>371411</v>
       </c>
-      <c r="F22" s="13" t="inlineStr"/>
       <c r="G22" s="13" t="inlineStr"/>
+      <c r="H22" s="13" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
@@ -1069,22 +1108,22 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A32:G32"/>
-    <mergeCell ref="A44:G44"/>
-    <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A34:G34"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="A46:G46"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A38:G38"/>
-    <mergeCell ref="A29:G29"/>
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A43:G43"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="A47:G47"/>
-    <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1096,7 +1135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1104,8 +1143,9 @@
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1136,10 +1176,15 @@
       </c>
       <c r="F1" s="20" t="inlineStr">
         <is>
+          <t>Net weight (kg)</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
           <t>Gross weight (kg)</t>
         </is>
       </c>
-      <c r="G1" s="20" t="inlineStr">
+      <c r="H1" s="20" t="inlineStr">
         <is>
           <t>Value (RMB)</t>
         </is>
@@ -1168,9 +1213,12 @@
         <v>972</v>
       </c>
       <c r="F2" s="4" t="n">
+        <v>769.5</v>
+      </c>
+      <c r="G2" s="4" t="n">
         <v>834.3</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>59292</v>
       </c>
     </row>
@@ -1197,9 +1245,12 @@
         <v>300</v>
       </c>
       <c r="F3" s="4" t="n">
+        <v>365</v>
+      </c>
+      <c r="G3" s="4" t="n">
         <v>395</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="H3" s="4" t="n">
         <v>35100</v>
       </c>
     </row>
@@ -1226,9 +1277,12 @@
         <v>762</v>
       </c>
       <c r="F4" s="4" t="n">
+        <v>635</v>
+      </c>
+      <c r="G4" s="4" t="n">
         <v>673.1</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>71628</v>
       </c>
     </row>
@@ -1255,9 +1309,12 @@
         <v>600</v>
       </c>
       <c r="F5" s="4" t="n">
+        <v>590</v>
+      </c>
+      <c r="G5" s="4" t="n">
         <v>630</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>51000</v>
       </c>
     </row>
@@ -1284,9 +1341,12 @@
         <v>156</v>
       </c>
       <c r="F6" s="4" t="n">
+        <v>221</v>
+      </c>
+      <c r="G6" s="4" t="n">
         <v>234</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>13728</v>
       </c>
     </row>
@@ -1313,9 +1373,12 @@
         <v>180</v>
       </c>
       <c r="F7" s="4" t="n">
+        <v>472.5</v>
+      </c>
+      <c r="G7" s="4" t="n">
         <v>508.5</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>14220</v>
       </c>
     </row>
@@ -1342,9 +1405,12 @@
         <v>300</v>
       </c>
       <c r="F8" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="G8" s="4" t="n">
         <v>320</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>4600</v>
       </c>
     </row>
@@ -1371,9 +1437,12 @@
         <v>354</v>
       </c>
       <c r="F9" s="4" t="n">
+        <v>684.4</v>
+      </c>
+      <c r="G9" s="4" t="n">
         <v>725.7</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>20532</v>
       </c>
     </row>
@@ -1400,9 +1469,12 @@
         <v>504</v>
       </c>
       <c r="F10" s="4" t="n">
+        <v>1243.2</v>
+      </c>
+      <c r="G10" s="4" t="n">
         <v>1293.6</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>36288</v>
       </c>
     </row>
@@ -1429,9 +1501,12 @@
         <v>210</v>
       </c>
       <c r="F11" s="4" t="n">
+        <v>168</v>
+      </c>
+      <c r="G11" s="4" t="n">
         <v>185.5</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>7980</v>
       </c>
     </row>
@@ -1458,9 +1533,12 @@
         <v>250</v>
       </c>
       <c r="F12" s="4" t="n">
+        <v>287.5</v>
+      </c>
+      <c r="G12" s="4" t="n">
         <v>302.5</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>8875</v>
       </c>
     </row>
@@ -1487,9 +1565,12 @@
         <v>180</v>
       </c>
       <c r="F13" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G13" s="4" t="n">
         <v>25.2</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="H13" s="4" t="n">
         <v>4770</v>
       </c>
     </row>
@@ -1516,9 +1597,12 @@
         <v>180</v>
       </c>
       <c r="F14" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>25.2</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>4230</v>
       </c>
     </row>
@@ -1545,9 +1629,12 @@
         <v>120</v>
       </c>
       <c r="F15" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="G15" s="4" t="n">
         <v>158</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="H15" s="4" t="n">
         <v>5520</v>
       </c>
     </row>
@@ -1574,9 +1661,12 @@
         <v>400</v>
       </c>
       <c r="F16" s="4" t="n">
+        <v>760</v>
+      </c>
+      <c r="G16" s="4" t="n">
         <v>820</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>15600</v>
       </c>
     </row>
@@ -1603,9 +1693,12 @@
         <v>168</v>
       </c>
       <c r="F17" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="G17" s="4" t="n">
         <v>104.5</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="H17" s="4" t="n">
         <v>17808</v>
       </c>
     </row>
@@ -1632,9 +1725,12 @@
         <v>30</v>
       </c>
       <c r="F18" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G18" s="4" t="n">
         <v>2.9</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="H18" s="4" t="n">
         <v>240</v>
       </c>
     </row>
@@ -1651,9 +1747,12 @@
         <v>5666</v>
       </c>
       <c r="F19" s="13" t="n">
+        <v>6795.7</v>
+      </c>
+      <c r="G19" s="13" t="n">
         <v>7238</v>
       </c>
-      <c r="G19" s="13" t="n">
+      <c r="H19" s="13" t="n">
         <v>371411</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Confirm antidumping duty on ironing board line (TARIC 7323990010)
Verified against TARIC and EUR-Lex: definitive AD duty on ironing
boards from China renewed by Implementing Regulation (EU) 2025/2386
(27-Nov-2025). Note 4 now lists company-specific rates and additional
codes; residual A999 rate 42.3% unless a listed producer is evidenced.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DEStrPTYqhj9hDeddsySih
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Fired_Up_OOCU5773452.xlsx
+++ b/output/HS_Code_Summary_Fired_Up_OOCU5773452.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t>Yes - verify</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1039,14 +1039,14 @@
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>4. ANTIDUMPING - ironing board (TARIC 7323990010):</t>
+          <t>4. ANTIDUMPING CONFIRMED - ironing board (TARIC 7323990010, item 4922):</t>
         </is>
       </c>
     </row>
     <row r="35" ht="42" customHeight="1">
       <c r="A35" s="18" t="inlineStr">
         <is>
-          <t>Item 4922 uses the TARIC add-on code for ironing boards from China, historically subject to EU anti-dumping duty (up to 42.3%, residual). Verify the current measure status in TARIC before clearance - the supplier's use of the ...10 code signals AD relevance.</t>
+          <t>Definitive anti-dumping duty on ironing boards from China, renewed 27-Nov-2025 by Commission Implementing Regulation (EU) 2025/2386 (TARIC measure D552, shown for CN with 'viz podminky'). Rate depends on the actual PRODUCER (TARIC additional code): A785 Guangdong Wireking 18.1%; A953 Greenwood Houseware 22.7%; A786 Zhejiang Harmonic 26.5%; A782 Foshan City Gaoming Lihe 34.9%; A784 Since Hardware 35.8%; A783 Guangzhou Power Team 39.6%; A999 ALL OTHER companies 42.3%. Supplier Fired Up Trading Co Ltd is not a listed producer - unless the manufacturer is identified as one of the named companies, declare A999 at 42.3% (approx. 3,754 RMB on the 8,875 RMB line) on top of the 3.2% conventional duty.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use Czech invoice descriptions as primary column in HS summary
Popis (CZ) taken verbatim from invoice column L is now the main
description on both sheets, with the English name kept as secondary.
CLAUDE.md updated so Czech descriptions and net weights are standing
rules for all future shipments.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DEStrPTYqhj9hDeddsySih
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Fired_Up_OOCU5773452.xlsx
+++ b/output/HS_Code_Summary_Fired_Up_OOCU5773452.xlsx
@@ -515,17 +515,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -627,35 +628,40 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Popis (CZ)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
+          <t>Description (EN)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
           <t>Total quantity (pcs)</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Net weight (kg)</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Gross weight (kg)</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Customs value (RMB)</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Antidumping</t>
         </is>
@@ -669,27 +675,32 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>Fén na vlasy</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
           <t>Hair dryers (Corby Milton 2000W)</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="D12" s="5" t="n">
         <v>972</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="E12" s="6" t="n">
         <v>769.5</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="F12" s="6" t="n">
         <v>834.3</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="G12" s="5" t="n">
         <v>59292</v>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -699,27 +710,32 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
+          <t>Rychlovarná konvice</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
           <t>Electric kettles (Hertford 1.8L; Kensington 0.6L; Double Walled 0.6L)</t>
         </is>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="D13" s="8" t="n">
         <v>1662</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="E13" s="9" t="n">
         <v>1590</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="F13" s="9" t="n">
         <v>1698.1</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="G13" s="8" t="n">
         <v>157728</v>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr"/>
+      <c r="I13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -729,27 +745,32 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>Pohlcovač plísní</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
           <t>Anti-mould device (electric space heating), steel, white</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="D14" s="5" t="n">
         <v>168</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="E14" s="6" t="n">
         <v>99</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="F14" s="6" t="n">
         <v>104.5</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="G14" s="5" t="n">
         <v>17808</v>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -759,27 +780,32 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
+          <t>Hotelové zrcadlo volně stojící</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
           <t>Framed glass mirror - free standing illuminated (Winchester)</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="D15" s="8" t="n">
         <v>156</v>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="E15" s="9" t="n">
         <v>221</v>
       </c>
-      <c r="E15" s="9" t="n">
+      <c r="F15" s="9" t="n">
         <v>234</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="G15" s="8" t="n">
         <v>13728</v>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr"/>
+      <c r="I15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -789,27 +815,32 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
+          <t>Odpadkový koš</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
           <t>Steel household bins / waste bins (Rectangular dual recycling; 9L double layer; Highland 9L; Newport 6+6L; Thornton 9L)</t>
         </is>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="D16" s="5" t="n">
         <v>1548</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="E16" s="6" t="n">
         <v>2868.1</v>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="F16" s="6" t="n">
         <v>3033.3</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="G16" s="5" t="n">
         <v>83620</v>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>No*</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -819,27 +850,32 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
+          <t>Žehlící prkno</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
           <t>Table top ironing board - dark grey</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
+      <c r="D17" s="11" t="n">
         <v>250</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="E17" s="12" t="n">
         <v>287.5</v>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="F17" s="12" t="n">
         <v>302.5</v>
       </c>
-      <c r="F17" s="11" t="n">
+      <c r="G17" s="11" t="n">
         <v>8875</v>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="H17" s="10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H17" s="10" t="inlineStr">
+      <c r="I17" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -853,27 +889,32 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
+          <t>Háček na oblečení</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
           <t>Steel double clothes hooks (Harrogate, black / polished)</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="D18" s="5" t="n">
         <v>360</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="E18" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="E18" s="6" t="n">
+      <c r="F18" s="6" t="n">
         <v>50.4</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="G18" s="5" t="n">
         <v>9000</v>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -883,27 +924,32 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
+          <t>Držák na zavazadla</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
           <t>Metal luggage racks (Ashton, black)</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="D19" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="D19" s="9" t="n">
+      <c r="E19" s="9" t="n">
         <v>760</v>
       </c>
-      <c r="E19" s="9" t="n">
+      <c r="F19" s="9" t="n">
         <v>820</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="G19" s="8" t="n">
         <v>15600</v>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr"/>
+      <c r="I19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -913,27 +959,32 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
+          <t>Obal na kapesníčky s povrchovou úpravou kůže</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
           <t>PU leather tissue box cover (CUBE)</t>
         </is>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="D20" s="5" t="n">
         <v>120</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="E20" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="E20" s="6" t="n">
+      <c r="F20" s="6" t="n">
         <v>158</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="G20" s="5" t="n">
         <v>5520</v>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -943,27 +994,32 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
+          <t>Propojovací kabel (viz pozn. 5)</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
           <t>Anti-mould device connector cable (supplier code - see note 5)</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="D21" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="D21" s="9" t="n">
+      <c r="E21" s="9" t="n">
         <v>2.6</v>
       </c>
-      <c r="E21" s="9" t="n">
+      <c r="F21" s="9" t="n">
         <v>2.9</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="G21" s="8" t="n">
         <v>240</v>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr"/>
+      <c r="I21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
@@ -972,20 +1028,21 @@
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr"/>
-      <c r="C22" s="14" t="n">
+      <c r="C22" s="13" t="inlineStr"/>
+      <c r="D22" s="14" t="n">
         <v>5666</v>
       </c>
-      <c r="D22" s="15" t="n">
+      <c r="E22" s="15" t="n">
         <v>6795.7</v>
       </c>
-      <c r="E22" s="15" t="n">
+      <c r="F22" s="15" t="n">
         <v>7238</v>
       </c>
-      <c r="F22" s="14" t="n">
+      <c r="G22" s="14" t="n">
         <v>371411</v>
       </c>
-      <c r="G22" s="13" t="inlineStr"/>
       <c r="H22" s="13" t="inlineStr"/>
+      <c r="I22" s="13" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
@@ -1108,22 +1165,22 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="A35:H35"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A40:H40"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A41:H41"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A37:I37"/>
+    <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A46:I46"/>
+    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A34:I34"/>
+    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A38:I38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1135,17 +1192,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1161,30 +1219,35 @@
       </c>
       <c r="C1" s="20" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Popis (CZ)</t>
         </is>
       </c>
       <c r="D1" s="20" t="inlineStr">
         <is>
+          <t>Description (EN)</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
           <t>HS code (invoice)</t>
         </is>
       </c>
-      <c r="E1" s="20" t="inlineStr">
+      <c r="F1" s="20" t="inlineStr">
         <is>
           <t>Qty (pcs)</t>
         </is>
       </c>
-      <c r="F1" s="20" t="inlineStr">
+      <c r="G1" s="20" t="inlineStr">
         <is>
           <t>Net weight (kg)</t>
         </is>
       </c>
-      <c r="G1" s="20" t="inlineStr">
+      <c r="H1" s="20" t="inlineStr">
         <is>
           <t>Gross weight (kg)</t>
         </is>
       </c>
-      <c r="H1" s="20" t="inlineStr">
+      <c r="I1" s="20" t="inlineStr">
         <is>
           <t>Value (RMB)</t>
         </is>
@@ -1201,24 +1264,29 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
+          <t>Fén na vlasy</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
           <t>Corby - Milton - 2000W Hair Dryer - Black - EU plug</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>8516310000</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="F2" s="4" t="n">
         <v>972</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="G2" s="4" t="n">
         <v>769.5</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>834.3</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>59292</v>
       </c>
     </row>
@@ -1233,24 +1301,29 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
+          <t>Rychlovarná konvice</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
           <t>Corby - Hertford - 1.8L Kettle - Black &amp; Chrome - EU Plug</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>8516797090</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="F3" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="G3" s="4" t="n">
         <v>365</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="H3" s="4" t="n">
         <v>395</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="I3" s="4" t="n">
         <v>35100</v>
       </c>
     </row>
@@ -1265,24 +1338,29 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
+          <t>Rychlovarná konvice</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
           <t>Corby - Kensington - 0.6L Kettle - Brushed Steel - EU Plug</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>8516797090</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="F4" s="4" t="n">
         <v>762</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="G4" s="4" t="n">
         <v>635</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>673.1</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>71628</v>
       </c>
     </row>
@@ -1297,24 +1375,29 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>Rychlovarná konvice</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
           <t>0.6L Double Walled Kettle - Black - EU plug</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>8516797090</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>600</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="G5" s="4" t="n">
         <v>590</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>630</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>51000</v>
       </c>
     </row>
@@ -1329,24 +1412,29 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
+          <t>Hotelové zrcadlo volně stojící</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
           <t>Corby - Winchester - Free Standing Illuminated Mirror - Chrome</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>7009920000</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>156</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="G6" s="4" t="n">
         <v>221</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>234</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>13728</v>
       </c>
     </row>
@@ -1361,24 +1449,29 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
+          <t>Odpadkový koš</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
           <t>Corby - Rectangular - Dual Recycling Bin - Plastic Inserts - Black</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>7323990090</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="G7" s="4" t="n">
         <v>472.5</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>508.5</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>14220</v>
       </c>
     </row>
@@ -1393,24 +1486,29 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
+          <t>Odpadkový koš</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
           <t>9L Double Layer Bin - Black (6 pcs/ctn)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>7323990090</t>
         </is>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>300</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>300</v>
       </c>
       <c r="G8" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="H8" s="4" t="n">
         <v>320</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>4600</v>
       </c>
     </row>
@@ -1425,24 +1523,29 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
+          <t>Odpadkový koš</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
           <t>Corby - Highland - 9L Double Layer Bin PU Leather - Black</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>7323990090</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>354</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="G9" s="4" t="n">
         <v>684.4</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>725.7</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="I9" s="4" t="n">
         <v>20532</v>
       </c>
     </row>
@@ -1457,24 +1560,29 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
+          <t>Odpadkový koš</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
           <t>Corby - Newport - 6+6L Bin - Black</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>7323990090</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>504</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="G10" s="4" t="n">
         <v>1243.2</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>1293.6</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="I10" s="4" t="n">
         <v>36288</v>
       </c>
     </row>
@@ -1489,24 +1597,29 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
+          <t>Odpadkový koš</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
           <t>Corby - Thornton - 9L Single Layer Bin - Brushed Steel (6 pcs/ctn)</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>7323990090</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="F11" s="4" t="n">
         <v>210</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="G11" s="4" t="n">
         <v>168</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>185.5</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="I11" s="4" t="n">
         <v>7980</v>
       </c>
     </row>
@@ -1521,24 +1634,29 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
+          <t>Žehlící prkno</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
           <t>Table Top Ironing Board - Dark Grey</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>7323990010</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>250</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="G12" s="4" t="n">
         <v>287.5</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>302.5</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>8875</v>
       </c>
     </row>
@@ -1553,24 +1671,29 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
+          <t>Háček na oblečení</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
           <t>Corby - Harrogate - Double Clothes Hook - Black</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>7324900090</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="F13" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="G13" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="H13" s="4" t="n">
         <v>25.2</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="I13" s="4" t="n">
         <v>4770</v>
       </c>
     </row>
@@ -1585,24 +1708,29 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
+          <t>Háček na oblečení</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
           <t>Corby - Harrogate - Double Clothes Hook - Polished Steel</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>7324900090</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>25.2</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="I14" s="4" t="n">
         <v>4230</v>
       </c>
     </row>
@@ -1617,24 +1745,29 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
+          <t>Obal na kapesníčky s povrchovou úpravou kůže</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
           <t>Corby - CUBE - PU Leather Tissue Box Cover - Black</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>3924900090</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="F15" s="4" t="n">
         <v>120</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="G15" s="4" t="n">
         <v>150</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="H15" s="4" t="n">
         <v>158</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="I15" s="4" t="n">
         <v>5520</v>
       </c>
     </row>
@@ -1649,24 +1782,29 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
+          <t>Držák na zavazadla</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
           <t>Corby - Ashton - Metal Luggage Rack - Black - No Back</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>9403208000</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="F16" s="4" t="n">
         <v>400</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="G16" s="4" t="n">
         <v>760</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>820</v>
       </c>
-      <c r="H16" s="4" t="n">
+      <c r="I16" s="4" t="n">
         <v>15600</v>
       </c>
     </row>
@@ -1681,24 +1819,29 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
+          <t>Pohlcovač plísní</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
           <t>Anti-Mould Device - Steel - White - EU Plug</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>8516299100</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="F17" s="4" t="n">
         <v>168</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="G17" s="4" t="n">
         <v>99</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="H17" s="4" t="n">
         <v>104.5</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="I17" s="4" t="n">
         <v>17808</v>
       </c>
     </row>
@@ -1713,46 +1856,52 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
+          <t>Propojovací kabel</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
           <t>Anti-Mould Device - Connector Cable</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>8708919990</t>
         </is>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="F18" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="G18" s="4" t="n">
         <v>2.6</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="H18" s="4" t="n">
         <v>2.9</v>
       </c>
-      <c r="H18" s="4" t="n">
+      <c r="I18" s="4" t="n">
         <v>240</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr"/>
       <c r="B19" s="13" t="inlineStr"/>
-      <c r="C19" s="13" t="inlineStr">
+      <c r="C19" s="13" t="inlineStr"/>
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D19" s="13" t="inlineStr"/>
-      <c r="E19" s="13" t="n">
+      <c r="E19" s="13" t="inlineStr"/>
+      <c r="F19" s="13" t="n">
         <v>5666</v>
       </c>
-      <c r="F19" s="13" t="n">
+      <c r="G19" s="13" t="n">
         <v>6795.7</v>
       </c>
-      <c r="G19" s="13" t="n">
+      <c r="H19" s="13" t="n">
         <v>7238</v>
       </c>
-      <c r="H19" s="13" t="n">
+      <c r="I19" s="13" t="n">
         <v>371411</v>
       </c>
     </row>

</xml_diff>